<commit_message>
feat: halaman KKT Unsrat Angkatan 149, tautan kredit di footer
- kkt.html: 15 mahasiswa KKT dikelompokkan per bidang (nama, NIM, fakultas,
  peran), data di DATA_KKT pada halaman/kkt.js, tidak ada di menu atas
- Footer: tautan "Dikembangkan oleh Mahasiswa KKT Unsrat Angkatan 149"
- visualOrang mendukung foto dari tab lain; kartu orang dibatasi lebarnya
- Batas wilayah di data contoh & template disamakan dengan spreadsheet
- README & panduan teknis mencatat halaman KKT

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/template-data-lahendong.xlsx
+++ b/data/template-data-lahendong.xlsx
@@ -2560,19 +2560,19 @@
     <t xml:space="preserve">CONTOH — ganti. Satuan °C. Profil.</t>
   </si>
   <si>
-    <t xml:space="preserve">Kelurahan Kampung Jawa</t>
+    <t xml:space="preserve">Tumatangtang 1, Kampung Jawa</t>
   </si>
   <si>
     <t xml:space="preserve">Profil, tabel batas wilayah.</t>
   </si>
   <si>
-    <t xml:space="preserve">Kabupaten Minahasa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kecamatan Pangolombian</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kelurahan Pinaras</t>
+    <t xml:space="preserve">Leilem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pangolombian, Tondangow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pinaras, Rambunan</t>
   </si>
   <si>
     <t xml:space="preserve">Lahendong tumbuh dari perkampungan kecil di sekitar sumber panas bumi alami di kaki pegunungan Tomohon.

</xml_diff>

<commit_message>
feat: kepala & wakil kepala lingkungan dalam satu kartu
- Tab lingkungan: kolom wakil_kepala; data kepala & wakil Lingkungan 1–6 dan 8,
  Lingkungan 7 kosong (tampil "Belum tersedia", juga bila sel terhapus)
- Kartu lingkungan baru: nomor, jiwa & KK, batang porsi, kepala dan wakil kepala
- Cek Data: nama tercatat di dua lingkungan/jabatan, kepala = wakil, jabatan kosong
- Template & panduan diperbarui

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/template-data-lahendong.xlsx
+++ b/data/template-data-lahendong.xlsx
@@ -169,7 +169,7 @@
               </xdr:from>
               <xdr:to>
                 <xdr:col>2</xdr:col>
-                <xdr:colOff>32</xdr:colOff>
+                <xdr:colOff>-76</xdr:colOff>
                 <xdr:row>7</xdr:row>
                 <xdr:rowOff>8</xdr:rowOff>
               </xdr:to>
@@ -187,8 +187,8 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Nama kepala lingkungan. Kosong = "Belum dicantumkan".
-Contoh: Nama lengkap</t>
+          <t xml:space="preserve">Nama KEPALA lingkungan di baris lingkungannya. Kosong = tampil "Belum tersedia".
+Contoh: Julius Joni Rondonuwu</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -203,9 +203,9 @@
               </xdr:from>
               <xdr:to>
                 <xdr:col>3</xdr:col>
-                <xdr:colOff>32</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>10</xdr:rowOff>
+                <xdr:colOff>-84</xdr:colOff>
+                <xdr:row>8</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -214,6 +214,40 @@
       </mc:AlternateContent>
     </comment>
     <comment ref="C1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Nama WAKIL kepala lingkungan di baris lingkungannya. Kosong = tampil "Belum tersedia".
+Contoh: Jetni Vinsensia Poli</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>23</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>32</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>3</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -230,13 +264,13 @@
           <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
-                <xdr:col>3</xdr:col>
+                <xdr:col>4</xdr:col>
                 <xdr:colOff>23</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>0</xdr:rowOff>
               </xdr:from>
               <xdr:to>
-                <xdr:col>4</xdr:col>
+                <xdr:col>5</xdr:col>
                 <xdr:colOff>32</xdr:colOff>
                 <xdr:row>3</xdr:row>
                 <xdr:rowOff>16</xdr:rowOff>
@@ -247,7 +281,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D1" authorId="0">
+    <comment ref="E1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -264,13 +298,13 @@
           <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
-                <xdr:col>4</xdr:col>
+                <xdr:col>5</xdr:col>
                 <xdr:colOff>23</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>0</xdr:rowOff>
               </xdr:from>
               <xdr:to>
-                <xdr:col>5</xdr:col>
+                <xdr:col>6</xdr:col>
                 <xdr:colOff>32</xdr:colOff>
                 <xdr:row>6</xdr:row>
                 <xdr:rowOff>10</xdr:rowOff>
@@ -281,7 +315,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="E1" authorId="0">
+    <comment ref="F1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -298,14 +332,14 @@
           <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
-                <xdr:col>5</xdr:col>
+                <xdr:col>6</xdr:col>
                 <xdr:colOff>23</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>0</xdr:rowOff>
               </xdr:from>
               <xdr:to>
-                <xdr:col>6</xdr:col>
-                <xdr:colOff>8</xdr:colOff>
+                <xdr:col>7</xdr:col>
+                <xdr:colOff>7</xdr:colOff>
                 <xdr:row>3</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -315,7 +349,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="F1" authorId="0">
+    <comment ref="G1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -332,13 +366,13 @@
           <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
-                <xdr:col>6</xdr:col>
+                <xdr:col>7</xdr:col>
                 <xdr:colOff>23</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>0</xdr:rowOff>
               </xdr:from>
               <xdr:to>
-                <xdr:col>7</xdr:col>
+                <xdr:col>8</xdr:col>
                 <xdr:colOff>16</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>3</xdr:rowOff>
@@ -349,7 +383,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="G1" authorId="0">
+    <comment ref="H1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -366,13 +400,13 @@
           <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
-                <xdr:col>7</xdr:col>
+                <xdr:col>8</xdr:col>
                 <xdr:colOff>23</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>0</xdr:rowOff>
               </xdr:from>
               <xdr:to>
-                <xdr:col>8</xdr:col>
+                <xdr:col>9</xdr:col>
                 <xdr:colOff>47</xdr:colOff>
                 <xdr:row>2</xdr:row>
                 <xdr:rowOff>3</xdr:rowOff>
@@ -1808,7 +1842,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="407">
   <si>
     <t xml:space="preserve">PETUNJUK MENGELOLA DATA — Website Kelurahan Lahendong</t>
   </si>
@@ -1882,7 +1916,7 @@
     <t xml:space="preserve">Penduduk (angka, grafik &amp; tabel), Beranda (angka ringkas), Pemerintahan (kartu lingkungan)</t>
   </si>
   <si>
-    <t xml:space="preserve">Satu baris per lingkungan. Semua total (penduduk, KK, jiwa) dihitung otomatis dari tab ini</t>
+    <t xml:space="preserve">Satu baris per lingkungan: kepala &amp; wakil kepala lingkungan, KK, laki-laki, perempuan, lansia, rumah. Semua total dihitung otomatis dari tab ini</t>
   </si>
   <si>
     <t xml:space="preserve">aparat</t>
@@ -2026,10 +2060,19 @@
     <t xml:space="preserve">lingkungan · kepala</t>
   </si>
   <si>
-    <t xml:space="preserve">Nama kepala lingkungan. Kosong = "Belum dicantumkan".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nama lengkap</t>
+    <t xml:space="preserve">Nama KEPALA lingkungan di baris lingkungannya. Kosong = tampil "Belum tersedia".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Julius Joni Rondonuwu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lingkungan · wakil_kepala</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nama WAKIL kepala lingkungan di baris lingkungannya. Kosong = tampil "Belum tersedia".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jetni Vinsensia Poli</t>
   </si>
   <si>
     <t xml:space="preserve">lingkungan · jumlah_kk</t>
@@ -2515,7 +2558,7 @@
     <t xml:space="preserve">• Tab layanan: syarat, alur, waktu, biaya, dan catatan setiap surat perlu dicocokkan dengan ketentuan kantor kelurahan.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Masih kosong: telepon_kantor, email, nama kepala lingkungan, nomor aparat, UMKM, galeri.</t>
+    <t xml:space="preserve">• Masih kosong: telepon_kantor, email, kepala &amp; wakil kepala Lingkungan 7, nomor aparat, UMKM, galeri.</t>
   </si>
   <si>
     <t xml:space="preserve">kunci</t>
@@ -2612,6 +2655,9 @@
     <t xml:space="preserve">kepala</t>
   </si>
   <si>
+    <t xml:space="preserve">wakil_kepala</t>
+  </si>
+  <si>
     <t xml:space="preserve">jumlah_kk</t>
   </si>
   <si>
@@ -2630,6 +2676,12 @@
     <t xml:space="preserve">Lingkungan 1</t>
   </si>
   <si>
+    <t xml:space="preserve">Jonathan Tombuku Londok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Femmi Selvie Kowel</t>
+  </si>
+  <si>
     <t xml:space="preserve">116</t>
   </si>
   <si>
@@ -2645,6 +2697,12 @@
     <t xml:space="preserve">80</t>
   </si>
   <si>
+    <t xml:space="preserve">Reynold Happy Sondakh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jefry Hengky Mende</t>
+  </si>
+  <si>
     <t xml:space="preserve">114</t>
   </si>
   <si>
@@ -2660,6 +2718,12 @@
     <t xml:space="preserve">Lingkungan 4</t>
   </si>
   <si>
+    <t xml:space="preserve">Djerry Andreu Legi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fredy Ali</t>
+  </si>
+  <si>
     <t xml:space="preserve">67</t>
   </si>
   <si>
@@ -2678,6 +2742,12 @@
     <t xml:space="preserve">Lingkungan 5</t>
   </si>
   <si>
+    <t xml:space="preserve">Tombuku Costan Sumolang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trully Treyse Lalawi</t>
+  </si>
+  <si>
     <t xml:space="preserve">113</t>
   </si>
   <si>
@@ -2696,6 +2766,12 @@
     <t xml:space="preserve">Lingkungan 6</t>
   </si>
   <si>
+    <t xml:space="preserve">Marho Katotje Singal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marten Singal</t>
+  </si>
+  <si>
     <t xml:space="preserve">96</t>
   </si>
   <si>
@@ -2727,6 +2803,12 @@
   </si>
   <si>
     <t xml:space="preserve">Lingkungan 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jon Junus Mende</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Treisye Roisye Rondonuwu</t>
   </si>
   <si>
     <t xml:space="preserve">97</t>
@@ -3342,7 +3424,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28.6"/>
@@ -3675,7 +3757,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
         <v>74</v>
       </c>
@@ -3731,28 +3813,28 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="4" t="s">
+      <c r="A55" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C55" s="4" t="s">
+      <c r="C55" s="2" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="2" t="s">
+      <c r="A56" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B56" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="C56" s="2" t="s">
+      <c r="C56" s="4" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
         <v>95</v>
       </c>
@@ -3763,7 +3845,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
         <v>98</v>
       </c>
@@ -3774,7 +3856,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
         <v>101</v>
       </c>
@@ -3785,25 +3867,25 @@
         <v>103</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="4" t="s">
+    <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="B60" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C60" s="4" t="s">
+      <c r="C60" s="2" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="2" t="s">
+      <c r="A61" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="B61" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="C61" s="2" t="s">
+      <c r="C61" s="4" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3841,47 +3923,47 @@
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="4" t="s">
+      <c r="A65" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B65" s="4" t="s">
+      <c r="B65" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="C65" s="4" t="s">
+      <c r="C65" s="2" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="2" t="s">
+      <c r="A66" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B66" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B66" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>125</v>
+        <v>105</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>126</v>
+        <v>106</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3973,47 +4055,47 @@
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="4" t="s">
+      <c r="A77" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="B77" s="4" t="s">
+      <c r="B77" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="C77" s="4" t="s">
+      <c r="C77" s="2" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="2" t="s">
+      <c r="A78" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="B78" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B78" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>157</v>
+        <v>105</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>158</v>
+        <v>106</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4024,51 +4106,51 @@
         <v>160</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>100</v>
+        <v>161</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>163</v>
+        <v>103</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="4" t="s">
+      <c r="A83" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="B83" s="4" t="s">
+      <c r="B83" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="C83" s="4" t="s">
+      <c r="C83" s="2" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="2" t="s">
+      <c r="A84" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="B84" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C84" s="2" t="s">
-        <v>109</v>
+      <c r="B84" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>169</v>
+        <v>111</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>170</v>
+        <v>112</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4127,237 +4209,248 @@
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="4" t="s">
+      <c r="A91" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="B91" s="4" t="s">
+      <c r="B91" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="C91" s="4" t="s">
+      <c r="C91" s="2" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="2" t="s">
+      <c r="A92" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="B92" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C92" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="93" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B92" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>191</v>
+        <v>111</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>194</v>
+        <v>106</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="2"/>
+      <c r="A95" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="3" t="s">
-        <v>195</v>
-      </c>
+      <c r="A96" s="2"/>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="B97" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="B98" s="3" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="B98" s="2" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>61</v>
+        <v>204</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>204</v>
+        <v>61</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="2"/>
-    </row>
-    <row r="115" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="3" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="116" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="2" t="s">
+      <c r="A114" s="2" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="117" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B114" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="2"/>
+    </row>
+    <row r="116" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="3" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="2" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="2"/>
+        <v>232</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="2" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="3" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="120" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="2" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="121" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="2"/>
+    </row>
+    <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="3" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="2" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="122" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="2" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="123" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="2" t="s">
-        <v>235</v>
+        <v>237</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="2" t="s">
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -4385,42 +4478,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4431,137 +4524,137 @@
         <v>64</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>254</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5081,43 +5174,50 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G109"/>
+  <dimension ref="A1:H109"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="13.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="29.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="13.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="15.73"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>270</v>
+        <v>273</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="B2" s="2"/>
+        <v>275</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>73</v>
+      </c>
       <c r="C2" s="2" t="s">
         <v>76</v>
       </c>
@@ -5133,152 +5233,186 @@
       <c r="G2" s="2" t="s">
         <v>88</v>
       </c>
+      <c r="H2" s="2" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="B3" s="2"/>
+        <v>166</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>276</v>
+      </c>
       <c r="C3" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>276</v>
+        <v>281</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>283</v>
+      </c>
       <c r="C4" s="2" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>280</v>
+        <v>287</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="B5" s="2"/>
+        <v>289</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>290</v>
+      </c>
       <c r="C5" s="2" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>285</v>
+        <v>294</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>286</v>
+        <v>295</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="B6" s="2"/>
+        <v>297</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>298</v>
+      </c>
       <c r="C6" s="2" t="s">
-        <v>288</v>
+        <v>299</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>289</v>
+        <v>300</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>290</v>
+        <v>301</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>291</v>
+        <v>302</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>292</v>
+        <v>303</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="B7" s="2"/>
+        <v>305</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>306</v>
+      </c>
       <c r="C7" s="2" t="s">
-        <v>294</v>
+        <v>307</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>296</v>
+        <v>309</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>298</v>
+        <v>311</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>299</v>
+        <v>313</v>
       </c>
       <c r="B8" s="2"/>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="2"/>
+      <c r="D8" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>302</v>
-      </c>
       <c r="G8" s="2" t="s">
-        <v>303</v>
+        <v>316</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="B9" s="2"/>
+        <v>318</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>319</v>
+      </c>
       <c r="C9" s="2" t="s">
-        <v>305</v>
+        <v>320</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>306</v>
+        <v>321</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>274</v>
+        <v>322</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>307</v>
+        <v>280</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>308</v>
+        <v>323</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5289,6 +5423,7 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2"/>
@@ -5298,6 +5433,7 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
@@ -5307,6 +5443,7 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2"/>
@@ -5316,6 +5453,7 @@
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2"/>
@@ -5325,6 +5463,7 @@
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2"/>
@@ -5334,6 +5473,7 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
@@ -5343,6 +5483,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2"/>
@@ -5352,6 +5493,7 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2"/>
@@ -5361,6 +5503,7 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2"/>
@@ -5370,6 +5513,7 @@
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2"/>
@@ -5379,6 +5523,7 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2"/>
@@ -5388,6 +5533,7 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2"/>
@@ -5397,6 +5543,7 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2"/>
@@ -5406,6 +5553,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2"/>
@@ -5415,6 +5563,7 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2"/>
@@ -5424,6 +5573,7 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2"/>
@@ -5433,6 +5583,7 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2"/>
@@ -5442,6 +5593,7 @@
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2"/>
@@ -5451,6 +5603,7 @@
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2"/>
@@ -5460,6 +5613,7 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2"/>
@@ -5469,6 +5623,7 @@
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2"/>
@@ -5478,6 +5633,7 @@
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2"/>
@@ -5487,6 +5643,7 @@
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2"/>
@@ -5496,6 +5653,7 @@
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2"/>
@@ -5505,6 +5663,7 @@
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2"/>
@@ -5514,6 +5673,7 @@
       <c r="E35" s="2"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2"/>
@@ -5523,6 +5683,7 @@
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2"/>
@@ -5532,6 +5693,7 @@
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2"/>
@@ -5541,6 +5703,7 @@
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2"/>
@@ -5550,6 +5713,7 @@
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2"/>
@@ -5559,6 +5723,7 @@
       <c r="E40" s="2"/>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2"/>
@@ -5568,6 +5733,7 @@
       <c r="E41" s="2"/>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2"/>
@@ -5577,6 +5743,7 @@
       <c r="E42" s="2"/>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2"/>
@@ -5586,6 +5753,7 @@
       <c r="E43" s="2"/>
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2"/>
@@ -5595,6 +5763,7 @@
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2"/>
@@ -5604,6 +5773,7 @@
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2"/>
@@ -5613,6 +5783,7 @@
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
+      <c r="H46" s="2"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2"/>
@@ -5622,6 +5793,7 @@
       <c r="E47" s="2"/>
       <c r="F47" s="2"/>
       <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2"/>
@@ -5631,6 +5803,7 @@
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2"/>
@@ -5640,6 +5813,7 @@
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
       <c r="G49" s="2"/>
+      <c r="H49" s="2"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2"/>
@@ -5649,6 +5823,7 @@
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
       <c r="G50" s="2"/>
+      <c r="H50" s="2"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2"/>
@@ -5658,6 +5833,7 @@
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
       <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2"/>
@@ -5667,6 +5843,7 @@
       <c r="E52" s="2"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
+      <c r="H52" s="2"/>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2"/>
@@ -5676,6 +5853,7 @@
       <c r="E53" s="2"/>
       <c r="F53" s="2"/>
       <c r="G53" s="2"/>
+      <c r="H53" s="2"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2"/>
@@ -5685,6 +5863,7 @@
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
+      <c r="H54" s="2"/>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2"/>
@@ -5694,6 +5873,7 @@
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
+      <c r="H55" s="2"/>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2"/>
@@ -5703,6 +5883,7 @@
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
+      <c r="H56" s="2"/>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2"/>
@@ -5712,6 +5893,7 @@
       <c r="E57" s="2"/>
       <c r="F57" s="2"/>
       <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2"/>
@@ -5721,6 +5903,7 @@
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
+      <c r="H58" s="2"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2"/>
@@ -5730,6 +5913,7 @@
       <c r="E59" s="2"/>
       <c r="F59" s="2"/>
       <c r="G59" s="2"/>
+      <c r="H59" s="2"/>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2"/>
@@ -5739,6 +5923,7 @@
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
+      <c r="H60" s="2"/>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2"/>
@@ -5748,6 +5933,7 @@
       <c r="E61" s="2"/>
       <c r="F61" s="2"/>
       <c r="G61" s="2"/>
+      <c r="H61" s="2"/>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2"/>
@@ -5757,6 +5943,7 @@
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
+      <c r="H62" s="2"/>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2"/>
@@ -5766,6 +5953,7 @@
       <c r="E63" s="2"/>
       <c r="F63" s="2"/>
       <c r="G63" s="2"/>
+      <c r="H63" s="2"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2"/>
@@ -5775,6 +5963,7 @@
       <c r="E64" s="2"/>
       <c r="F64" s="2"/>
       <c r="G64" s="2"/>
+      <c r="H64" s="2"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2"/>
@@ -5784,6 +5973,7 @@
       <c r="E65" s="2"/>
       <c r="F65" s="2"/>
       <c r="G65" s="2"/>
+      <c r="H65" s="2"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2"/>
@@ -5793,6 +5983,7 @@
       <c r="E66" s="2"/>
       <c r="F66" s="2"/>
       <c r="G66" s="2"/>
+      <c r="H66" s="2"/>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2"/>
@@ -5802,6 +5993,7 @@
       <c r="E67" s="2"/>
       <c r="F67" s="2"/>
       <c r="G67" s="2"/>
+      <c r="H67" s="2"/>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2"/>
@@ -5811,6 +6003,7 @@
       <c r="E68" s="2"/>
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
+      <c r="H68" s="2"/>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2"/>
@@ -5820,6 +6013,7 @@
       <c r="E69" s="2"/>
       <c r="F69" s="2"/>
       <c r="G69" s="2"/>
+      <c r="H69" s="2"/>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2"/>
@@ -5829,6 +6023,7 @@
       <c r="E70" s="2"/>
       <c r="F70" s="2"/>
       <c r="G70" s="2"/>
+      <c r="H70" s="2"/>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2"/>
@@ -5838,6 +6033,7 @@
       <c r="E71" s="2"/>
       <c r="F71" s="2"/>
       <c r="G71" s="2"/>
+      <c r="H71" s="2"/>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2"/>
@@ -5847,6 +6043,7 @@
       <c r="E72" s="2"/>
       <c r="F72" s="2"/>
       <c r="G72" s="2"/>
+      <c r="H72" s="2"/>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2"/>
@@ -5856,6 +6053,7 @@
       <c r="E73" s="2"/>
       <c r="F73" s="2"/>
       <c r="G73" s="2"/>
+      <c r="H73" s="2"/>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2"/>
@@ -5865,6 +6063,7 @@
       <c r="E74" s="2"/>
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
+      <c r="H74" s="2"/>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2"/>
@@ -5874,6 +6073,7 @@
       <c r="E75" s="2"/>
       <c r="F75" s="2"/>
       <c r="G75" s="2"/>
+      <c r="H75" s="2"/>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2"/>
@@ -5883,6 +6083,7 @@
       <c r="E76" s="2"/>
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
+      <c r="H76" s="2"/>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2"/>
@@ -5892,6 +6093,7 @@
       <c r="E77" s="2"/>
       <c r="F77" s="2"/>
       <c r="G77" s="2"/>
+      <c r="H77" s="2"/>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2"/>
@@ -5901,6 +6103,7 @@
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
+      <c r="H78" s="2"/>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2"/>
@@ -5910,6 +6113,7 @@
       <c r="E79" s="2"/>
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
+      <c r="H79" s="2"/>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2"/>
@@ -5919,6 +6123,7 @@
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
+      <c r="H80" s="2"/>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2"/>
@@ -5928,6 +6133,7 @@
       <c r="E81" s="2"/>
       <c r="F81" s="2"/>
       <c r="G81" s="2"/>
+      <c r="H81" s="2"/>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2"/>
@@ -5937,6 +6143,7 @@
       <c r="E82" s="2"/>
       <c r="F82" s="2"/>
       <c r="G82" s="2"/>
+      <c r="H82" s="2"/>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2"/>
@@ -5946,6 +6153,7 @@
       <c r="E83" s="2"/>
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
+      <c r="H83" s="2"/>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2"/>
@@ -5955,6 +6163,7 @@
       <c r="E84" s="2"/>
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>
+      <c r="H84" s="2"/>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2"/>
@@ -5964,6 +6173,7 @@
       <c r="E85" s="2"/>
       <c r="F85" s="2"/>
       <c r="G85" s="2"/>
+      <c r="H85" s="2"/>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2"/>
@@ -5973,6 +6183,7 @@
       <c r="E86" s="2"/>
       <c r="F86" s="2"/>
       <c r="G86" s="2"/>
+      <c r="H86" s="2"/>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2"/>
@@ -5982,6 +6193,7 @@
       <c r="E87" s="2"/>
       <c r="F87" s="2"/>
       <c r="G87" s="2"/>
+      <c r="H87" s="2"/>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2"/>
@@ -5991,6 +6203,7 @@
       <c r="E88" s="2"/>
       <c r="F88" s="2"/>
       <c r="G88" s="2"/>
+      <c r="H88" s="2"/>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2"/>
@@ -6000,6 +6213,7 @@
       <c r="E89" s="2"/>
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
+      <c r="H89" s="2"/>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2"/>
@@ -6009,6 +6223,7 @@
       <c r="E90" s="2"/>
       <c r="F90" s="2"/>
       <c r="G90" s="2"/>
+      <c r="H90" s="2"/>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2"/>
@@ -6018,6 +6233,7 @@
       <c r="E91" s="2"/>
       <c r="F91" s="2"/>
       <c r="G91" s="2"/>
+      <c r="H91" s="2"/>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2"/>
@@ -6027,6 +6243,7 @@
       <c r="E92" s="2"/>
       <c r="F92" s="2"/>
       <c r="G92" s="2"/>
+      <c r="H92" s="2"/>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2"/>
@@ -6036,6 +6253,7 @@
       <c r="E93" s="2"/>
       <c r="F93" s="2"/>
       <c r="G93" s="2"/>
+      <c r="H93" s="2"/>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2"/>
@@ -6045,6 +6263,7 @@
       <c r="E94" s="2"/>
       <c r="F94" s="2"/>
       <c r="G94" s="2"/>
+      <c r="H94" s="2"/>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2"/>
@@ -6054,6 +6273,7 @@
       <c r="E95" s="2"/>
       <c r="F95" s="2"/>
       <c r="G95" s="2"/>
+      <c r="H95" s="2"/>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2"/>
@@ -6063,6 +6283,7 @@
       <c r="E96" s="2"/>
       <c r="F96" s="2"/>
       <c r="G96" s="2"/>
+      <c r="H96" s="2"/>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2"/>
@@ -6072,6 +6293,7 @@
       <c r="E97" s="2"/>
       <c r="F97" s="2"/>
       <c r="G97" s="2"/>
+      <c r="H97" s="2"/>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2"/>
@@ -6081,6 +6303,7 @@
       <c r="E98" s="2"/>
       <c r="F98" s="2"/>
       <c r="G98" s="2"/>
+      <c r="H98" s="2"/>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2"/>
@@ -6090,6 +6313,7 @@
       <c r="E99" s="2"/>
       <c r="F99" s="2"/>
       <c r="G99" s="2"/>
+      <c r="H99" s="2"/>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2"/>
@@ -6099,6 +6323,7 @@
       <c r="E100" s="2"/>
       <c r="F100" s="2"/>
       <c r="G100" s="2"/>
+      <c r="H100" s="2"/>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2"/>
@@ -6108,6 +6333,7 @@
       <c r="E101" s="2"/>
       <c r="F101" s="2"/>
       <c r="G101" s="2"/>
+      <c r="H101" s="2"/>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2"/>
@@ -6117,6 +6343,7 @@
       <c r="E102" s="2"/>
       <c r="F102" s="2"/>
       <c r="G102" s="2"/>
+      <c r="H102" s="2"/>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2"/>
@@ -6126,6 +6353,7 @@
       <c r="E103" s="2"/>
       <c r="F103" s="2"/>
       <c r="G103" s="2"/>
+      <c r="H103" s="2"/>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2"/>
@@ -6135,6 +6363,7 @@
       <c r="E104" s="2"/>
       <c r="F104" s="2"/>
       <c r="G104" s="2"/>
+      <c r="H104" s="2"/>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2"/>
@@ -6144,6 +6373,7 @@
       <c r="E105" s="2"/>
       <c r="F105" s="2"/>
       <c r="G105" s="2"/>
+      <c r="H105" s="2"/>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2"/>
@@ -6153,6 +6383,7 @@
       <c r="E106" s="2"/>
       <c r="F106" s="2"/>
       <c r="G106" s="2"/>
+      <c r="H106" s="2"/>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2"/>
@@ -6162,6 +6393,7 @@
       <c r="E107" s="2"/>
       <c r="F107" s="2"/>
       <c r="G107" s="2"/>
+      <c r="H107" s="2"/>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2"/>
@@ -6171,6 +6403,7 @@
       <c r="E108" s="2"/>
       <c r="F108" s="2"/>
       <c r="G108" s="2"/>
+      <c r="H108" s="2"/>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2"/>
@@ -6180,6 +6413,7 @@
       <c r="E109" s="2"/>
       <c r="F109" s="2"/>
       <c r="G109" s="2"/>
+      <c r="H109" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -6208,27 +6442,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>309</v>
+        <v>325</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>310</v>
+        <v>326</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>311</v>
+        <v>327</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>312</v>
+        <v>328</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="2"/>
@@ -6236,26 +6470,26 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>314</v>
+        <v>330</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>315</v>
+        <v>331</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -6994,70 +7228,70 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>311</v>
+        <v>327</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>318</v>
+        <v>334</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>319</v>
+        <v>335</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>320</v>
+        <v>336</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>321</v>
+        <v>337</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>322</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>323</v>
+        <v>339</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>324</v>
+        <v>340</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>322</v>
+        <v>338</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>325</v>
+        <v>341</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>326</v>
+        <v>342</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>327</v>
+        <v>343</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>322</v>
+        <v>338</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7800,144 +8034,144 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>312</v>
+        <v>328</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>328</v>
+        <v>344</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>329</v>
+        <v>345</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>330</v>
+        <v>346</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>331</v>
+        <v>347</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>332</v>
+        <v>348</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>333</v>
+        <v>349</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>334</v>
+        <v>350</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>335</v>
+        <v>351</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>336</v>
+        <v>352</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="s">
-        <v>337</v>
+        <v>353</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>338</v>
+        <v>354</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>339</v>
+        <v>355</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>340</v>
+        <v>356</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>341</v>
+        <v>357</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>342</v>
+        <v>358</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>343</v>
+        <v>359</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>344</v>
+        <v>360</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>345</v>
+        <v>361</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>346</v>
+        <v>362</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2" t="s">
-        <v>347</v>
+        <v>363</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>348</v>
+        <v>364</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>349</v>
+        <v>365</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>350</v>
+        <v>366</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>351</v>
+        <v>367</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>352</v>
+        <v>368</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>353</v>
+        <v>369</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>354</v>
+        <v>370</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>355</v>
+        <v>371</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>356</v>
+        <v>372</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
-        <v>357</v>
+        <v>373</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>358</v>
+        <v>374</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>359</v>
+        <v>375</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>360</v>
+        <v>376</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>361</v>
+        <v>377</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>362</v>
+        <v>378</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2" t="s">
-        <v>363</v>
+        <v>379</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9371,16 +9605,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>312</v>
+        <v>328</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>364</v>
+        <v>380</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>28</v>
@@ -10231,149 +10465,149 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>365</v>
+        <v>381</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>318</v>
+        <v>334</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>366</v>
+        <v>382</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>367</v>
+        <v>383</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>368</v>
+        <v>384</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>369</v>
+        <v>385</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>370</v>
+        <v>386</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>371</v>
+        <v>387</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>372</v>
+        <v>388</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>373</v>
+        <v>389</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>374</v>
+        <v>390</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="H2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>375</v>
+        <v>391</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>376</v>
+        <v>392</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>377</v>
+        <v>393</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>378</v>
+        <v>394</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>379</v>
+        <v>395</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>372</v>
+        <v>388</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>380</v>
+        <v>396</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>381</v>
+        <v>397</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="H4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>382</v>
+        <v>398</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>383</v>
+        <v>399</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>384</v>
+        <v>400</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>385</v>
+        <v>401</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>386</v>
+        <v>402</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="H5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>387</v>
+        <v>403</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>372</v>
+        <v>388</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>388</v>
+        <v>404</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>389</v>
+        <v>405</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="H6" s="2"/>
     </row>
@@ -11412,16 +11646,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>390</v>
+        <v>406</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>312</v>
+        <v>328</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>318</v>
+        <v>334</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
refactor: hapus halaman UMKM dan Legenda
- Hapus umkm.html, legenda.html, skrip, dan gambar legenda; keluarkan dari menu
- Hapus tab umkm & kunci profil legenda dari SKEMA, data contoh, template, Cek Data
- Galeri kini berisi foto tab galeri + foto wisata
- Perbarui README, DESIGN-SPEC, panduan admin & teknis

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/template-data-lahendong.xlsx
+++ b/data/template-data-lahendong.xlsx
@@ -14,9 +14,8 @@
     <sheet name="aparat" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="kontak" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="wisata" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="umkm" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="layanan" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="galeri" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="layanan" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="galeri" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -1213,220 +1212,6 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">WAJIB. Nama usaha. Untuk menghapus usaha: hapus barisnya.
-Contoh: Kue Lapis Bu Ani</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>23</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>32</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>10</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="B1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Ya = tampil di situs. Tidak = disembunyikan, data tetap tersimpan. Kosong dianggap Ya.
-Contoh: Ya</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>23</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>32</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="C1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Opsional. Tautan berbagi Google Drive satu foto (Bagikan → Siapa saja yang memiliki link → Salin link). Kosong = foto bawaan situs.
-Contoh: https://drive.google.com/file/d/…/view</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>23</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>4</xdr:col>
-                <xdr:colOff>32</xdr:colOff>
-                <xdr:row>11</xdr:row>
-                <xdr:rowOff>14</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="D1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Produk utama.
-Contoh: Kue lapis legit, kue kering</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>4</xdr:col>
-                <xdr:colOff>23</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>5</xdr:col>
-                <xdr:colOff>32</xdr:colOff>
-                <xdr:row>3</xdr:row>
-                <xdr:rowOff>16</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="E1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Nomor telepon/WA usaha — hanya bila pemilik setuju ditampilkan.
-Contoh: 0812-3456-7890</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>5</xdr:col>
-                <xdr:colOff>23</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>6</xdr:col>
-                <xdr:colOff>32</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="F1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Lokasi usaha, pilih dari daftar (diambil dari tab lingkungan).
-Contoh: Lingkungan 2</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>6</xdr:col>
-                <xdr:colOff>23</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>7</xdr:col>
-                <xdr:colOff>47</xdr:colOff>
-                <xdr:row>5</xdr:row>
-                <xdr:rowOff>12</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
-  <authors>
-    <author> </author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
           <t xml:space="preserve">WAJIB. Nama surat. Untuk menghapus surat: hapus barisnya.
 Contoh: Surat Keterangan Tidak Mampu (SKTM)</t>
         </r>
@@ -1695,7 +1480,7 @@
 </comments>
 </file>
 
-<file path=xl/comments9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author> </author>
@@ -1842,7 +1627,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="387">
   <si>
     <t xml:space="preserve">PETUNJUK MENGELOLA DATA — Website Kelurahan Lahendong</t>
   </si>
@@ -1904,10 +1689,10 @@
     <t xml:space="preserve">profil</t>
   </si>
   <si>
-    <t xml:space="preserve">Profil, Legenda, Kontak, Layanan, Penduduk (tahun &amp; sumber), Beranda (foto besar), header &amp; footer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alamat, telepon, email &amp; jam layanan kantor; luas, ketinggian, suhu; batas wilayah; sejarah; legenda; tahun &amp; sumber data; foto hero</t>
+    <t xml:space="preserve">Profil, Kontak, Layanan, Penduduk (tahun &amp; sumber), Beranda (foto besar), header &amp; footer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alamat, telepon, email &amp; jam layanan kantor; luas, ketinggian, suhu; batas wilayah; sejarah; tahun &amp; sumber data; foto hero</t>
   </si>
   <si>
     <t xml:space="preserve">lingkungan</t>
@@ -1946,15 +1731,6 @@
     <t xml:space="preserve">Satu baris per destinasi</t>
   </si>
   <si>
-    <t xml:space="preserve">umkm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UMKM, Galeri</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Satu baris per usaha</t>
-  </si>
-  <si>
     <t xml:space="preserve">layanan</t>
   </si>
   <si>
@@ -1970,7 +1746,7 @@
     <t xml:space="preserve">Galeri</t>
   </si>
   <si>
-    <t xml:space="preserve">Foto tambahan (kegiatan, alam, budaya) selain foto wisata &amp; UMKM</t>
+    <t xml:space="preserve">Foto tambahan (kegiatan, alam, budaya) selain foto wisata</t>
   </si>
   <si>
     <t xml:space="preserve">ATURAN PENGISIAN</t>
@@ -2306,45 +2082,6 @@
     <t xml:space="preserve">https://maps.google.com/?q=Danau+Linow</t>
   </si>
   <si>
-    <t xml:space="preserve">umkm · nama</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WAJIB. Nama usaha. Untuk menghapus usaha: hapus barisnya.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kue Lapis Bu Ani</t>
-  </si>
-  <si>
-    <t xml:space="preserve">umkm · tampil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">umkm · foto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">umkm · produk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Produk utama.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kue lapis legit, kue kering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">umkm · kontak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nomor telepon/WA usaha — hanya bila pemilik setuju ditampilkan.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">umkm · lingkungan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lokasi usaha, pilih dari daftar (diambil dari tab lingkungan).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lingkungan 2</t>
-  </si>
-  <si>
     <t xml:space="preserve">layanan · nama_surat</t>
   </si>
   <si>
@@ -2513,12 +2250,6 @@
     <t xml:space="preserve">Sejarah, satu paragraf per baris</t>
   </si>
   <si>
-    <t xml:space="preserve">legenda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legenda Danau Linow, satu paragraf per baris</t>
-  </si>
-  <si>
     <t xml:space="preserve">tahun_data</t>
   </si>
   <si>
@@ -2552,13 +2283,13 @@
     <t xml:space="preserve">Nilai yang belum ada data resminya ditandai "CONTOH" di kolom keterangan dan wajib diganti sebelum situs diumumkan:</t>
   </si>
   <si>
-    <t xml:space="preserve">• Tab profil: jam_layanan, luas_wilayah, ketinggian, suhu, sejarah, legenda.</t>
+    <t xml:space="preserve">• Tab profil: jam_layanan, luas_wilayah, ketinggian, suhu, sejarah.</t>
   </si>
   <si>
     <t xml:space="preserve">• Tab layanan: syarat, alur, waktu, biaya, dan catatan setiap surat perlu dicocokkan dengan ketentuan kantor kelurahan.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Masih kosong: telepon_kantor, email, kepala &amp; wakil kepala Lingkungan 7, nomor aparat, UMKM, galeri.</t>
+    <t xml:space="preserve">• Masih kosong: telepon_kantor, email, kepala &amp; wakil kepala Lingkungan 7, nomor aparat, galeri.</t>
   </si>
   <si>
     <t xml:space="preserve">kunci</t>
@@ -2626,14 +2357,6 @@
     <t xml:space="preserve">CONTOH — ganti. Profil. Satu baris dalam sel = satu paragraf; paragraf pertama ditampilkan lebih besar.</t>
   </si>
   <si>
-    <t xml:space="preserve">Warga percaya kawasan Danau Linow adalah tempat bersemayamnya roh penjaga alam, dan uap belerang yang terus mengepul adalah napasnya.
-Cerita turun-temurun menyebutkan bahwa warna air danau yang berubah-ubah adalah pertanda suasana hati sang penjaga. Saat air berwarna cerah, warga meyakini alam sedang tenang dan hasil panen akan melimpah.
-Secara ilmiah, perubahan warna air danau dipengaruhi kandungan mineral dan aktivitas vulkanik di dasar danau. Namun kisah rakyat ini tetap diwariskan sebagai bagian dari kekayaan budaya setempat.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONTOH — ganti dengan cerita yang dituturkan warga. Halaman Legenda. Satu baris dalam sel = satu paragraf.</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026</t>
   </si>
   <si>
@@ -2674,6 +2397,9 @@
   </si>
   <si>
     <t xml:space="preserve">Lingkungan 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lingkungan 2</t>
   </si>
   <si>
     <t xml:space="preserve">Jonathan Tombuku Londok</t>
@@ -3002,9 +2728,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://maps.google.com/?q=Mahwatu+Tomohon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">produk</t>
   </si>
   <si>
     <t xml:space="preserve">nama_surat</t>
@@ -3424,7 +3147,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28.6"/>
@@ -3610,106 +3333,106 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="2"/>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B28" s="2" t="s">
+    </row>
+    <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C28" s="2" t="s">
+    </row>
+    <row r="31" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2"/>
-    </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
+    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="s">
+    <row r="33" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
+    <row r="34" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
+    <row r="35" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="s">
         <v>46</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2" t="s">
+    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
+    <row r="40" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2" t="s">
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2"/>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="3" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C43" s="3" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="3" t="s">
+    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C44" s="3" t="s">
+      <c r="C44" s="4" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="4" t="s">
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="B45" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C45" s="4" t="s">
+      <c r="C45" s="2" t="s">
         <v>61</v>
       </c>
     </row>
@@ -3725,28 +3448,28 @@
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="2" t="s">
+      <c r="A47" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C47" s="2" t="s">
+      <c r="C47" s="4" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="4" t="s">
+      <c r="A48" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B48" s="4" t="s">
+      <c r="B48" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C48" s="4" t="s">
+      <c r="C48" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
         <v>71</v>
       </c>
@@ -3757,7 +3480,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
         <v>74</v>
       </c>
@@ -3813,28 +3536,28 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="2" t="s">
+      <c r="A55" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B55" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C55" s="2" t="s">
+      <c r="C55" s="4" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="4" t="s">
+      <c r="A56" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C56" s="4" t="s">
+      <c r="C56" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
         <v>95</v>
       </c>
@@ -3845,7 +3568,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
         <v>98</v>
       </c>
@@ -3856,7 +3579,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
         <v>101</v>
       </c>
@@ -3867,25 +3590,25 @@
         <v>103</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="2" t="s">
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C60" s="2" t="s">
+      <c r="C60" s="4" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="4" t="s">
+      <c r="A61" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B61" s="4" t="s">
+      <c r="B61" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="C61" s="4" t="s">
+      <c r="C61" s="2" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3923,47 +3646,47 @@
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="2" t="s">
+      <c r="A65" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C65" s="2" t="s">
+      <c r="C65" s="4" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="4" t="s">
+      <c r="A66" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B66" s="4" t="s">
+      <c r="B66" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C66" s="4" t="s">
+      <c r="B67" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="2" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="2" t="s">
+      <c r="B68" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B67" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="2" t="s">
+      <c r="C68" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4055,402 +3778,317 @@
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="2" t="s">
+      <c r="A77" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="B77" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="C77" s="2" t="s">
+      <c r="C77" s="4" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="4" t="s">
+      <c r="A78" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="B78" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C78" s="4" t="s">
-        <v>156</v>
+      <c r="B78" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C79" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="B79" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
         <v>158</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>105</v>
+        <v>159</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>106</v>
+        <v>160</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>103</v>
+        <v>166</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="B84" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="C84" s="4" t="s">
-        <v>169</v>
+      <c r="A84" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>112</v>
+      <c r="A85" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>172</v>
+        <v>108</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>176</v>
+        <v>103</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="B89" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="C89" s="2" t="s">
+      <c r="A89" s="2"/>
+    </row>
+    <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="3" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="2" t="s">
+    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="B90" s="2" t="s">
+      <c r="B91" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="C90" s="2" t="s">
+      <c r="B92" s="2" t="s">
         <v>185</v>
-      </c>
-    </row>
-    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="B91" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="C91" s="2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="B92" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="C92" s="4" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C93" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="C94" s="2" t="s">
-        <v>106</v>
+        <v>189</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="B95" s="2" t="s">
+      <c r="B98" s="2" t="s">
         <v>196</v>
-      </c>
-      <c r="C95" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="2"/>
-    </row>
-    <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="3" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="B98" s="3" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>61</v>
+        <v>203</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="2"/>
+    </row>
+    <row r="108" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="B106" s="2" t="s">
+    </row>
+    <row r="109" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="2" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="2" t="s">
+    <row r="110" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B107" s="2" t="s">
+    </row>
+    <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="2"/>
+    </row>
+    <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="3" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="2" t="s">
+    <row r="113" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B108" s="2" t="s">
+    </row>
+    <row r="114" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="2" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="2" t="s">
+    <row r="115" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="B109" s="2" t="s">
+    </row>
+    <row r="116" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="2" t="s">
         <v>220</v>
-      </c>
-    </row>
-    <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="B110" s="2" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="B111" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="B112" s="2" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="B113" s="2" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="B114" s="2" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="2"/>
-    </row>
-    <row r="116" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="3" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="117" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="2" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="118" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="2" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="2"/>
-    </row>
-    <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="3" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="121" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="2" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="122" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="2" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="123" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="2" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="124" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="2" t="s">
-        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -4469,7 +4107,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.98"/>
@@ -4478,184 +4116,178 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>239</v>
+        <v>221</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>241</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>200</v>
+        <v>184</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>242</v>
+        <v>224</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>243</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>202</v>
+        <v>186</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>244</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>204</v>
+        <v>188</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>245</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>64</v>
-      </c>
       <c r="C5" s="2" t="s">
-        <v>246</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>207</v>
+        <v>191</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>247</v>
+        <v>229</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>248</v>
+        <v>230</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>209</v>
+        <v>193</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>249</v>
+        <v>231</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>250</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>211</v>
+        <v>195</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>251</v>
+        <v>233</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>252</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>253</v>
+        <v>235</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>254</v>
+        <v>236</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>255</v>
+        <v>237</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>254</v>
+        <v>236</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>254</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>219</v>
+        <v>203</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>257</v>
+        <v>239</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>254</v>
+        <v>236</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>221</v>
+        <v>205</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>258</v>
+        <v>240</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>223</v>
+        <v>207</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>260</v>
+        <v>242</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>261</v>
+        <v>243</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>225</v>
+        <v>209</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>262</v>
+        <v>244</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>264</v>
-      </c>
+        <v>211</v>
+      </c>
+      <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
-        <v>229</v>
-      </c>
+        <v>246</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2"/>
       <c r="B17" s="2"/>
-      <c r="C17" s="2" t="s">
-        <v>266</v>
-      </c>
+      <c r="C17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2"/>
@@ -5151,11 +4783,6 @@
       <c r="A116" s="2"/>
       <c r="B116" s="2"/>
       <c r="C116" s="2"/>
-    </row>
-    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="2"/>
-      <c r="B117" s="2"/>
-      <c r="C117" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -5187,232 +4814,232 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>267</v>
+        <v>247</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>268</v>
+        <v>248</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>269</v>
+        <v>249</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>271</v>
+        <v>251</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>272</v>
+        <v>252</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>273</v>
+        <v>253</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>274</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>275</v>
+        <v>255</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>166</v>
+        <v>256</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>276</v>
+        <v>257</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>277</v>
+        <v>258</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>278</v>
+        <v>259</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>279</v>
+        <v>260</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>280</v>
+        <v>261</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>281</v>
+        <v>262</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>282</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>283</v>
+        <v>264</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>284</v>
+        <v>265</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>282</v>
+        <v>263</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>285</v>
+        <v>266</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>286</v>
+        <v>267</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>287</v>
+        <v>268</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>288</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>289</v>
+        <v>270</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>290</v>
+        <v>271</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>291</v>
+        <v>272</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>293</v>
+        <v>274</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>294</v>
+        <v>275</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>295</v>
+        <v>276</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>296</v>
+        <v>277</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>297</v>
+        <v>278</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>298</v>
+        <v>279</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>299</v>
+        <v>280</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>300</v>
+        <v>281</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>301</v>
+        <v>282</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>302</v>
+        <v>283</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>303</v>
+        <v>284</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>304</v>
+        <v>285</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>305</v>
+        <v>286</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>306</v>
+        <v>287</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>307</v>
+        <v>288</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>308</v>
+        <v>289</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>309</v>
+        <v>290</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>310</v>
+        <v>291</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>311</v>
+        <v>292</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>312</v>
+        <v>293</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>313</v>
+        <v>294</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
-        <v>314</v>
+        <v>295</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>315</v>
+        <v>296</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>300</v>
+        <v>281</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>316</v>
+        <v>297</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>317</v>
+        <v>298</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>318</v>
+        <v>299</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>319</v>
+        <v>300</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>320</v>
+        <v>301</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>321</v>
+        <v>302</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>322</v>
+        <v>303</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>280</v>
+        <v>261</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>323</v>
+        <v>304</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>324</v>
+        <v>305</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6442,27 +6069,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>325</v>
+        <v>306</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>267</v>
+        <v>247</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>326</v>
+        <v>307</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>327</v>
+        <v>308</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>328</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="2"/>
@@ -6470,26 +6097,26 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>329</v>
+        <v>310</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>330</v>
+        <v>311</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>331</v>
+        <v>312</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -7228,70 +6855,70 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>267</v>
+        <v>247</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>332</v>
+        <v>313</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>333</v>
+        <v>314</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>327</v>
+        <v>308</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>334</v>
+        <v>315</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>335</v>
+        <v>316</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>336</v>
+        <v>317</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>337</v>
+        <v>318</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>338</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>339</v>
+        <v>320</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>340</v>
+        <v>321</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>300</v>
+        <v>281</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>338</v>
+        <v>319</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>341</v>
+        <v>322</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>342</v>
+        <v>323</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>343</v>
+        <v>324</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>338</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8034,144 +7661,144 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>267</v>
+        <v>247</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>344</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>345</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>346</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>347</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>348</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>349</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>350</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>351</v>
-      </c>
       <c r="L1" s="3" t="s">
-        <v>352</v>
+        <v>333</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="s">
-        <v>353</v>
+        <v>334</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>354</v>
+        <v>335</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>355</v>
+        <v>336</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>356</v>
+        <v>337</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>357</v>
+        <v>338</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>358</v>
+        <v>339</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>359</v>
+        <v>340</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>360</v>
+        <v>341</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>361</v>
+        <v>342</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>362</v>
+        <v>343</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2" t="s">
-        <v>363</v>
+        <v>344</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>364</v>
+        <v>345</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>365</v>
+        <v>346</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>366</v>
+        <v>347</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>367</v>
+        <v>348</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>368</v>
+        <v>349</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>369</v>
+        <v>350</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>370</v>
+        <v>351</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>371</v>
+        <v>352</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>372</v>
+        <v>353</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
-        <v>373</v>
+        <v>354</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>374</v>
+        <v>355</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>375</v>
+        <v>356</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>376</v>
+        <v>357</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>377</v>
+        <v>358</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>378</v>
+        <v>359</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2" t="s">
-        <v>379</v>
+        <v>360</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9597,859 +9224,6 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="1" style="0" width="13.49"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
-        <v>267</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>332</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>380</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="6"/>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="6"/>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="6"/>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="6"/>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="6"/>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="6"/>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="6"/>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="6"/>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="6"/>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="6"/>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="6"/>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="6"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="6"/>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="6"/>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="6"/>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2"/>
-      <c r="B17" s="6"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="6"/>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2"/>
-      <c r="B18" s="6"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="6"/>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2"/>
-      <c r="B19" s="6"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="6"/>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2"/>
-      <c r="B20" s="6"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="6"/>
-    </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2"/>
-      <c r="B21" s="6"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="6"/>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2"/>
-      <c r="B22" s="6"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="6"/>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2"/>
-      <c r="B23" s="6"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="6"/>
-    </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2"/>
-      <c r="B24" s="6"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="6"/>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2"/>
-      <c r="B25" s="6"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="6"/>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2"/>
-      <c r="B26" s="6"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="6"/>
-    </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2"/>
-      <c r="B27" s="6"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="6"/>
-    </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2"/>
-      <c r="B28" s="6"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="6"/>
-    </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2"/>
-      <c r="B29" s="6"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="6"/>
-    </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2"/>
-      <c r="B30" s="6"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="6"/>
-    </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2"/>
-      <c r="B31" s="6"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="6"/>
-    </row>
-    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2"/>
-      <c r="B32" s="6"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="6"/>
-    </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2"/>
-      <c r="B33" s="6"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="6"/>
-    </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2"/>
-      <c r="B34" s="6"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="6"/>
-    </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2"/>
-      <c r="B35" s="6"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="6"/>
-    </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2"/>
-      <c r="B36" s="6"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="6"/>
-    </row>
-    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2"/>
-      <c r="B37" s="6"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="6"/>
-    </row>
-    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2"/>
-      <c r="B38" s="6"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="6"/>
-    </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2"/>
-      <c r="B39" s="6"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="6"/>
-    </row>
-    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2"/>
-      <c r="B40" s="6"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="6"/>
-    </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="2"/>
-      <c r="B41" s="6"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="6"/>
-    </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="2"/>
-      <c r="B42" s="6"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="6"/>
-    </row>
-    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="2"/>
-      <c r="B43" s="6"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-      <c r="F43" s="6"/>
-    </row>
-    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="2"/>
-      <c r="B44" s="6"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="6"/>
-    </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="2"/>
-      <c r="B45" s="6"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="6"/>
-    </row>
-    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="2"/>
-      <c r="B46" s="6"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="6"/>
-    </row>
-    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="2"/>
-      <c r="B47" s="6"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="6"/>
-    </row>
-    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="2"/>
-      <c r="B48" s="6"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
-      <c r="F48" s="6"/>
-    </row>
-    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="2"/>
-      <c r="B49" s="6"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
-      <c r="F49" s="6"/>
-    </row>
-    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="2"/>
-      <c r="B50" s="6"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-      <c r="E50" s="2"/>
-      <c r="F50" s="6"/>
-    </row>
-    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="2"/>
-      <c r="B51" s="6"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="6"/>
-    </row>
-    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="2"/>
-      <c r="B52" s="6"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="6"/>
-    </row>
-    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="2"/>
-      <c r="B53" s="6"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="6"/>
-    </row>
-    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="2"/>
-      <c r="B54" s="6"/>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
-      <c r="F54" s="6"/>
-    </row>
-    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="2"/>
-      <c r="B55" s="6"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
-      <c r="E55" s="2"/>
-      <c r="F55" s="6"/>
-    </row>
-    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="2"/>
-      <c r="B56" s="6"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
-      <c r="F56" s="6"/>
-    </row>
-    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="2"/>
-      <c r="B57" s="6"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
-      <c r="F57" s="6"/>
-    </row>
-    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="2"/>
-      <c r="B58" s="6"/>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
-      <c r="E58" s="2"/>
-      <c r="F58" s="6"/>
-    </row>
-    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="2"/>
-      <c r="B59" s="6"/>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
-      <c r="E59" s="2"/>
-      <c r="F59" s="6"/>
-    </row>
-    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="2"/>
-      <c r="B60" s="6"/>
-      <c r="C60" s="2"/>
-      <c r="D60" s="2"/>
-      <c r="E60" s="2"/>
-      <c r="F60" s="6"/>
-    </row>
-    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="2"/>
-      <c r="B61" s="6"/>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-      <c r="E61" s="2"/>
-      <c r="F61" s="6"/>
-    </row>
-    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="2"/>
-      <c r="B62" s="6"/>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-      <c r="E62" s="2"/>
-      <c r="F62" s="6"/>
-    </row>
-    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="2"/>
-      <c r="B63" s="6"/>
-      <c r="C63" s="2"/>
-      <c r="D63" s="2"/>
-      <c r="E63" s="2"/>
-      <c r="F63" s="6"/>
-    </row>
-    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="2"/>
-      <c r="B64" s="6"/>
-      <c r="C64" s="2"/>
-      <c r="D64" s="2"/>
-      <c r="E64" s="2"/>
-      <c r="F64" s="6"/>
-    </row>
-    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="2"/>
-      <c r="B65" s="6"/>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-      <c r="E65" s="2"/>
-      <c r="F65" s="6"/>
-    </row>
-    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="2"/>
-      <c r="B66" s="6"/>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2"/>
-      <c r="E66" s="2"/>
-      <c r="F66" s="6"/>
-    </row>
-    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="2"/>
-      <c r="B67" s="6"/>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2"/>
-      <c r="E67" s="2"/>
-      <c r="F67" s="6"/>
-    </row>
-    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="2"/>
-      <c r="B68" s="6"/>
-      <c r="C68" s="2"/>
-      <c r="D68" s="2"/>
-      <c r="E68" s="2"/>
-      <c r="F68" s="6"/>
-    </row>
-    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="2"/>
-      <c r="B69" s="6"/>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
-      <c r="E69" s="2"/>
-      <c r="F69" s="6"/>
-    </row>
-    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="2"/>
-      <c r="B70" s="6"/>
-      <c r="C70" s="2"/>
-      <c r="D70" s="2"/>
-      <c r="E70" s="2"/>
-      <c r="F70" s="6"/>
-    </row>
-    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="2"/>
-      <c r="B71" s="6"/>
-      <c r="C71" s="2"/>
-      <c r="D71" s="2"/>
-      <c r="E71" s="2"/>
-      <c r="F71" s="6"/>
-    </row>
-    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="2"/>
-      <c r="B72" s="6"/>
-      <c r="C72" s="2"/>
-      <c r="D72" s="2"/>
-      <c r="E72" s="2"/>
-      <c r="F72" s="6"/>
-    </row>
-    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="2"/>
-      <c r="B73" s="6"/>
-      <c r="C73" s="2"/>
-      <c r="D73" s="2"/>
-      <c r="E73" s="2"/>
-      <c r="F73" s="6"/>
-    </row>
-    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="2"/>
-      <c r="B74" s="6"/>
-      <c r="C74" s="2"/>
-      <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
-      <c r="F74" s="6"/>
-    </row>
-    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="2"/>
-      <c r="B75" s="6"/>
-      <c r="C75" s="2"/>
-      <c r="D75" s="2"/>
-      <c r="E75" s="2"/>
-      <c r="F75" s="6"/>
-    </row>
-    <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="2"/>
-      <c r="B76" s="6"/>
-      <c r="C76" s="2"/>
-      <c r="D76" s="2"/>
-      <c r="E76" s="2"/>
-      <c r="F76" s="6"/>
-    </row>
-    <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="2"/>
-      <c r="B77" s="6"/>
-      <c r="C77" s="2"/>
-      <c r="D77" s="2"/>
-      <c r="E77" s="2"/>
-      <c r="F77" s="6"/>
-    </row>
-    <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="2"/>
-      <c r="B78" s="6"/>
-      <c r="C78" s="2"/>
-      <c r="D78" s="2"/>
-      <c r="E78" s="2"/>
-      <c r="F78" s="6"/>
-    </row>
-    <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="2"/>
-      <c r="B79" s="6"/>
-      <c r="C79" s="2"/>
-      <c r="D79" s="2"/>
-      <c r="E79" s="2"/>
-      <c r="F79" s="6"/>
-    </row>
-    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="2"/>
-      <c r="B80" s="6"/>
-      <c r="C80" s="2"/>
-      <c r="D80" s="2"/>
-      <c r="E80" s="2"/>
-      <c r="F80" s="6"/>
-    </row>
-    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="2"/>
-      <c r="B81" s="6"/>
-      <c r="C81" s="2"/>
-      <c r="D81" s="2"/>
-      <c r="E81" s="2"/>
-      <c r="F81" s="6"/>
-    </row>
-    <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="2"/>
-      <c r="B82" s="6"/>
-      <c r="C82" s="2"/>
-      <c r="D82" s="2"/>
-      <c r="E82" s="2"/>
-      <c r="F82" s="6"/>
-    </row>
-    <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="2"/>
-      <c r="B83" s="6"/>
-      <c r="C83" s="2"/>
-      <c r="D83" s="2"/>
-      <c r="E83" s="2"/>
-      <c r="F83" s="6"/>
-    </row>
-    <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="2"/>
-      <c r="B84" s="6"/>
-      <c r="C84" s="2"/>
-      <c r="D84" s="2"/>
-      <c r="E84" s="2"/>
-      <c r="F84" s="6"/>
-    </row>
-    <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="2"/>
-      <c r="B85" s="6"/>
-      <c r="C85" s="2"/>
-      <c r="D85" s="2"/>
-      <c r="E85" s="2"/>
-      <c r="F85" s="6"/>
-    </row>
-    <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="2"/>
-      <c r="B86" s="6"/>
-      <c r="C86" s="2"/>
-      <c r="D86" s="2"/>
-      <c r="E86" s="2"/>
-      <c r="F86" s="6"/>
-    </row>
-    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="2"/>
-      <c r="B87" s="6"/>
-      <c r="C87" s="2"/>
-      <c r="D87" s="2"/>
-      <c r="E87" s="2"/>
-      <c r="F87" s="6"/>
-    </row>
-    <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="2"/>
-      <c r="B88" s="6"/>
-      <c r="C88" s="2"/>
-      <c r="D88" s="2"/>
-      <c r="E88" s="2"/>
-      <c r="F88" s="6"/>
-    </row>
-    <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="2"/>
-      <c r="B89" s="6"/>
-      <c r="C89" s="2"/>
-      <c r="D89" s="2"/>
-      <c r="E89" s="2"/>
-      <c r="F89" s="6"/>
-    </row>
-    <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="2"/>
-      <c r="B90" s="6"/>
-      <c r="C90" s="2"/>
-      <c r="D90" s="2"/>
-      <c r="E90" s="2"/>
-      <c r="F90" s="6"/>
-    </row>
-    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="2"/>
-      <c r="B91" s="6"/>
-      <c r="C91" s="2"/>
-      <c r="D91" s="2"/>
-      <c r="E91" s="2"/>
-      <c r="F91" s="6"/>
-    </row>
-    <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="2"/>
-      <c r="B92" s="6"/>
-      <c r="C92" s="2"/>
-      <c r="D92" s="2"/>
-      <c r="E92" s="2"/>
-      <c r="F92" s="6"/>
-    </row>
-    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="2"/>
-      <c r="B93" s="6"/>
-      <c r="C93" s="2"/>
-      <c r="D93" s="2"/>
-      <c r="E93" s="2"/>
-      <c r="F93" s="6"/>
-    </row>
-    <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="2"/>
-      <c r="B94" s="6"/>
-      <c r="C94" s="2"/>
-      <c r="D94" s="2"/>
-      <c r="E94" s="2"/>
-      <c r="F94" s="6"/>
-    </row>
-    <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="2"/>
-      <c r="B95" s="6"/>
-      <c r="C95" s="2"/>
-      <c r="D95" s="2"/>
-      <c r="E95" s="2"/>
-      <c r="F95" s="6"/>
-    </row>
-    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="2"/>
-      <c r="B96" s="6"/>
-      <c r="C96" s="2"/>
-      <c r="D96" s="2"/>
-      <c r="E96" s="2"/>
-      <c r="F96" s="6"/>
-    </row>
-    <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="2"/>
-      <c r="B97" s="6"/>
-      <c r="C97" s="2"/>
-      <c r="D97" s="2"/>
-      <c r="E97" s="2"/>
-      <c r="F97" s="6"/>
-    </row>
-    <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="2"/>
-      <c r="B98" s="6"/>
-      <c r="C98" s="2"/>
-      <c r="D98" s="2"/>
-      <c r="E98" s="2"/>
-      <c r="F98" s="6"/>
-    </row>
-    <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="2"/>
-      <c r="B99" s="6"/>
-      <c r="C99" s="2"/>
-      <c r="D99" s="2"/>
-      <c r="E99" s="2"/>
-      <c r="F99" s="6"/>
-    </row>
-    <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="2"/>
-      <c r="B100" s="6"/>
-      <c r="C100" s="2"/>
-      <c r="D100" s="2"/>
-      <c r="E100" s="2"/>
-      <c r="F100" s="6"/>
-    </row>
-    <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="2"/>
-      <c r="B101" s="6"/>
-      <c r="C101" s="2"/>
-      <c r="D101" s="2"/>
-      <c r="E101" s="2"/>
-      <c r="F101" s="6"/>
-    </row>
-  </sheetData>
-  <dataValidations count="2">
-    <dataValidation allowBlank="true" error="Pilih salah satu dari daftar." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B101" type="list">
-      <formula1>"Ya,Tidak"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Pilih salah satu dari daftar." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F101" type="list">
-      <formula1>lingkungan!$A$2:$A$500</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
-  </headerFooter>
-  <legacyDrawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
   <dimension ref="A1:H106"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -10465,149 +9239,149 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>381</v>
+        <v>361</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>332</v>
+        <v>313</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>334</v>
+        <v>315</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>382</v>
+        <v>362</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>383</v>
+        <v>363</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>384</v>
+        <v>364</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>385</v>
+        <v>365</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>386</v>
+        <v>366</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>387</v>
+        <v>367</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>388</v>
+        <v>368</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>389</v>
+        <v>369</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>390</v>
+        <v>370</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>185</v>
+        <v>169</v>
       </c>
       <c r="H2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>185</v>
-      </c>
       <c r="H3" s="2" t="s">
-        <v>394</v>
+        <v>374</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>395</v>
+        <v>375</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>388</v>
+        <v>368</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>396</v>
+        <v>376</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>397</v>
+        <v>377</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>185</v>
+        <v>169</v>
       </c>
       <c r="H4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>398</v>
+        <v>378</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>399</v>
+        <v>379</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>400</v>
+        <v>380</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>401</v>
+        <v>381</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>402</v>
+        <v>382</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>185</v>
+        <v>169</v>
       </c>
       <c r="H5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>403</v>
+        <v>383</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>388</v>
+        <v>368</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>404</v>
+        <v>384</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>405</v>
+        <v>385</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>185</v>
+        <v>169</v>
       </c>
       <c r="H6" s="2"/>
     </row>
@@ -11633,7 +10407,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -11646,16 +10420,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>406</v>
+        <v>386</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>332</v>
+        <v>313</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>328</v>
+        <v>309</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>334</v>
+        <v>315</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
feat: foto dinamis dari folder Google Drive
- tools/sinkron-foto.gs: Apps Script membuat folder "Foto Situs Lahendong", membagikan
  foto, dan menulis isinya ke tab foto tiap 10 menit (menu Situs)
- Situs mengenali foto dari nama berkas & subfolder: beranda/hero, wisata/<nama>,
  aparat/<jabatan|nama>, lingkungan/<nama>, kkt/<NIM|nama>, galeri/<kategori>/<judul>
- Urutan sumber: kolom foto → folder Drive → img/ → pengganti/monogram
- Galeri otomatis memuat foto folder galeri/ dengan kategori dari subfolder
- Cek Data: nama berkas tak cocok (dengan saran), folder salah, nama ganda, foto tak terbuka
- Dokumentasi & template diperbarui

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/template-data-lahendong.xlsx
+++ b/data/template-data-lahendong.xlsx
@@ -570,7 +570,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Opsional. Tautan berbagi Google Drive satu foto (Bagikan → Siapa saja yang memiliki link → Salin link). Kosong = foto bawaan situs.
+          <t xml:space="preserve">Opsional — biasanya cukup unggah foto ke folder foto Drive dengan nama yang sesuai (lihat tab petunjuk). Isi kolom ini hanya untuk menimpanya dengan tautan berbagi satu foto.
 Contoh: https://drive.google.com/file/d/…/view</t>
         </r>
       </text>
@@ -587,8 +587,8 @@
               <xdr:to>
                 <xdr:col>6</xdr:col>
                 <xdr:colOff>47</xdr:colOff>
-                <xdr:row>11</xdr:row>
-                <xdr:rowOff>14</xdr:rowOff>
+                <xdr:row>16</xdr:row>
+                <xdr:rowOff>3</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -862,7 +862,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Opsional. Tautan berbagi Google Drive satu foto (Bagikan → Siapa saja yang memiliki link → Salin link). Kosong = foto bawaan situs.
+          <t xml:space="preserve">Opsional — biasanya cukup unggah foto ke folder foto Drive dengan nama yang sesuai (lihat tab petunjuk). Isi kolom ini hanya untuk menimpanya dengan tautan berbagi satu foto.
 Contoh: https://drive.google.com/file/d/…/view</t>
         </r>
       </text>
@@ -880,7 +880,7 @@
                 <xdr:col>4</xdr:col>
                 <xdr:colOff>-367</xdr:colOff>
                 <xdr:row>2</xdr:row>
-                <xdr:rowOff>33</xdr:rowOff>
+                <xdr:rowOff>108</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1562,7 +1562,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">WAJIB untuk galeri. Tautan berbagi Google Drive satu foto (Bagikan → Siapa saja yang memiliki link → Salin link).
+          <t xml:space="preserve">Tautan satu foto Drive — atau kosongkan dan unggah foto ke folder Drive galeri/ dengan nama berkas = judul.
 Contoh: https://drive.google.com/file/d/…/view</t>
         </r>
       </text>
@@ -1627,7 +1627,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="394">
   <si>
     <t xml:space="preserve">PETUNJUK MENGELOLA DATA — Website Kelurahan Lahendong</t>
   </si>
@@ -1659,22 +1659,37 @@
     <t xml:space="preserve">• Setelah mengubah data, buka halaman Cek Data: https://vercoooo.github.io/web-lahendong/cek-data.html — setiap isian yang keliru ditunjukkan beserta cara memperbaikinya.</t>
   </si>
   <si>
-    <t xml:space="preserve">FOTO DARI GOOGLE DRIVE (kolom foto &amp; kunci foto_hero)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Unggah foto (JPG/PNG, sisi terpanjang sekitar 1600 piksel sudah cukup) ke folder Google Drive situs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Klik kanan foto → Bagikan → Akses umum: "Siapa saja yang memiliki link" sebagai Pelihat. (Atur sekali di folder agar semua foto di dalamnya ikut.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Klik kanan foto → Bagikan → Salin link, lalu tempel di kolom foto pada baris yang sesuai.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Buka halaman Cek Data: foto yang belum dibagikan atau tautannya salah akan ditandai.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Gunakan tautan satu foto, bukan tautan folder. Foto orang hanya dengan izin yang bersangkutan.</t>
+    <t xml:space="preserve">FOTO DARI GOOGLE DRIVE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cara utama: unggah foto ke folder "Foto Situs Lahendong" di Google Drive (menu Situs → Buka folder foto). Situs mengenali foto dari NAMA BERKAS dan SUBFOLDER-nya:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• beranda/hero.jpg → gambar besar di Beranda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• wisata/&lt;nama destinasi&gt;.jpg → mis. wisata/Danau Linow.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• aparat/&lt;jabatan atau nama tanpa gelar&gt;.jpg → mis. aparat/Lurah.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• lingkungan/&lt;nama kepala/wakil&gt;.jpg → mis. lingkungan/Julius Joni Rondonuwu.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• kkt/&lt;NIM atau nama&gt;.jpg → mis. kkt/230211060074.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• galeri/&lt;kategori&gt;/&lt;judul&gt;.jpg → setiap foto otomatis masuk Galeri, mis. galeri/Kegiatan/Panen Raya.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mengganti foto: hapus berkas lama, unggah yang baru dengan nama sama. Menghapus: hapus berkasnya. Huruf besar/kecil dan ekstensi (.jpg/.png/.webp) bebas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perubahan tampil paling lambat 10 menit kemudian, atau segera lewat menu Situs → Sinkronkan foto sekarang. Foto orang 3:4 (pas foto), lanskap 3:2; hanya dengan izin yang bersangkutan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kolom foto di tab lain (tautan Drive satu foto) tetap bisa dipakai untuk menimpa foto dari folder. Cek Data menandai nama berkas yang tidak cocok dengan data mana pun.</t>
   </si>
   <si>
     <t xml:space="preserve">TAB</t>
@@ -1746,7 +1761,16 @@
     <t xml:space="preserve">Galeri</t>
   </si>
   <si>
-    <t xml:space="preserve">Foto tambahan (kegiatan, alam, budaya) selain foto wisata</t>
+    <t xml:space="preserve">Opsional: judul &amp; kategori lewat sheet. Foto di folder Drive galeri/ sudah otomatis masuk Galeri tanpa baris di sini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">foto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semua halaman yang berfoto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diisi OTOMATIS dari folder foto Google Drive oleh skrip (menu Situs). Jangan diedit.</t>
   </si>
   <si>
     <t xml:space="preserve">ATURAN PENGISIAN</t>
@@ -1935,7 +1959,7 @@
     <t xml:space="preserve">aparat · foto</t>
   </si>
   <si>
-    <t xml:space="preserve">Opsional. Tautan berbagi Google Drive satu foto (Bagikan → Siapa saja yang memiliki link → Salin link). Kosong = foto bawaan situs.</t>
+    <t xml:space="preserve">Opsional — biasanya cukup unggah foto ke folder foto Drive dengan nama yang sesuai (lihat tab petunjuk). Isi kolom ini hanya untuk menimpanya dengan tautan berbagi satu foto.</t>
   </si>
   <si>
     <t xml:space="preserve">https://drive.google.com/file/d/…/view</t>
@@ -2163,7 +2187,7 @@
     <t xml:space="preserve">galeri · foto</t>
   </si>
   <si>
-    <t xml:space="preserve">WAJIB untuk galeri. Tautan berbagi Google Drive satu foto (Bagikan → Siapa saja yang memiliki link → Salin link).</t>
+    <t xml:space="preserve">Tautan satu foto Drive — atau kosongkan dan unggah foto ke folder Drive galeri/ dengan nama berkas = judul.</t>
   </si>
   <si>
     <t xml:space="preserve">galeri · kategori</t>
@@ -2556,9 +2580,6 @@
   </si>
   <si>
     <t xml:space="preserve">nomor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">foto</t>
   </si>
   <si>
     <t xml:space="preserve">Sekretaris Kelurahan</t>
@@ -3147,7 +3168,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C122"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28.6"/>
@@ -3211,718 +3232,705 @@
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2"/>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="3" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="3" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
+    <row r="22" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="2" t="s">
+    </row>
+    <row r="23" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="2" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2"/>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="B25" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C25" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="2" t="s">
+    </row>
+    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+      <c r="B26" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="2" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+      <c r="B27" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="C27" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C24" s="2" t="s">
+    </row>
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+      <c r="B28" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C25" s="2" t="s">
+    </row>
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+      <c r="B29" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C29" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="2" t="s">
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
+      <c r="B30" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C27" s="2" t="s">
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2"/>
-    </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
+      <c r="B31" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
+      <c r="C31" s="2" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C32" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="35" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2" t="s">
+      <c r="B33" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="36" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C33" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="2"/>
-    </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="3" t="s">
+    </row>
+    <row r="41" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C43" s="3" t="s">
+    </row>
+    <row r="42" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="4" t="s">
+    <row r="43" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B44" s="4" t="s">
+    </row>
+    <row r="44" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C44" s="4" t="s">
+    </row>
+    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="2" t="s">
+    <row r="46" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B45" s="2" t="s">
+    </row>
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="2"/>
+    </row>
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C45" s="2" t="s">
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="3" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="2" t="s">
+      <c r="B49" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="C49" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C46" s="2" t="s">
+    </row>
+    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="4" t="s">
+      <c r="B50" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="C50" s="4" t="s">
         <v>66</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>85</v>
+      <c r="A53" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>91</v>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B61" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="C61" s="4" t="s">
         <v>99</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="C60" s="4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B67" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="C67" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="B65" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="C65" s="4" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>135</v>
+      <c r="A71" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>137</v>
+        <v>116</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>141</v>
+        <v>111</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="B77" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="C77" s="4" t="s">
-        <v>153</v>
+      <c r="A77" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>108</v>
+        <v>145</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>109</v>
+        <v>146</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>169</v>
+      <c r="A83" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>171</v>
+        <v>116</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>172</v>
+        <v>117</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="B85" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="C85" s="4" t="s">
-        <v>175</v>
+      <c r="A85" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>108</v>
+        <v>167</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>103</v>
+        <v>171</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B90" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="B88" s="2" t="s">
+      <c r="C90" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="C88" s="2" t="s">
+    </row>
+    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="4" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="2"/>
-    </row>
-    <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="3" t="s">
+      <c r="B91" s="4" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="3" t="s">
+      <c r="C91" s="4" t="s">
         <v>183</v>
-      </c>
-      <c r="B91" s="3" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3930,165 +3938,214 @@
         <v>184</v>
       </c>
       <c r="B92" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="2" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="2" t="s">
+      <c r="B93" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="B93" s="2" t="s">
-        <v>187</v>
+      <c r="C93" s="2" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B94" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B94" s="2" t="s">
+      <c r="C94" s="2" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B95" s="2" t="s">
+      <c r="A95" s="2"/>
+    </row>
+    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="3" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="2" t="s">
+    <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="B96" s="2" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="B97" s="2" t="s">
-        <v>194</v>
+      <c r="B97" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>201</v>
+        <v>66</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="B106" s="2" t="s">
+      <c r="B108" s="2" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="2"/>
-    </row>
-    <row r="108" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="3" t="s">
+    <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="2" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="109" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="2" t="s">
+      <c r="B109" s="2" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="2" t="s">
         <v>215</v>
       </c>
+      <c r="B110" s="2" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="2"/>
+      <c r="A111" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>218</v>
+      </c>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="3" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="113" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="2" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="114" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="2" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="115" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="2"/>
+    </row>
+    <row r="114" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="3" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="2" t="s">
-        <v>220</v>
+        <v>223</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="2"/>
+    </row>
+    <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="3" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="2" t="s">
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -4116,172 +4173,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4814,232 +4871,232 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6069,27 +6126,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>309</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="2"/>
@@ -6097,26 +6154,26 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -6855,70 +6912,70 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7661,144 +7718,144 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>309</v>
+        <v>45</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2" t="s">
-        <v>360</v>
+        <v>367</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9239,149 +9296,149 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>366</v>
+        <v>373</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="H2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>371</v>
+        <v>378</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>368</v>
-      </c>
       <c r="D4" s="2" t="s">
-        <v>376</v>
+        <v>383</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="H4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="H5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="H6" s="2"/>
     </row>
@@ -10420,16 +10477,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>309</v>
+        <v>45</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
feat: panel "Pasang / ganti foto" di spreadsheet menggantikan aturan nama berkas
- Cabut sistem folder Drive + pencocokan nama berkas (c668801): kode situs kembali
  sama dengan checkpoint-sebelum-gambar-dinamis
- tools/panel-foto.gs: pilih baris → menu Situs → Pasang / ganti foto → Simpan;
  foto diperkecil, disimpan ke Drive, dibagikan, tautannya ditulis ke kolom foto
- README, panduan admin & teknis, tab petunjuk template diperbarui

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/template-data-lahendong.xlsx
+++ b/data/template-data-lahendong.xlsx
@@ -570,7 +570,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Opsional — biasanya cukup unggah foto ke folder foto Drive dengan nama yang sesuai (lihat tab petunjuk). Isi kolom ini hanya untuk menimpanya dengan tautan berbagi satu foto.
+          <t xml:space="preserve">Diisi otomatis lewat menu Situs → Pasang / ganti foto (pilih barisnya dulu). Kosong = foto bawaan situs.
 Contoh: https://drive.google.com/file/d/…/view</t>
         </r>
       </text>
@@ -587,8 +587,8 @@
               <xdr:to>
                 <xdr:col>6</xdr:col>
                 <xdr:colOff>47</xdr:colOff>
-                <xdr:row>16</xdr:row>
-                <xdr:rowOff>3</xdr:rowOff>
+                <xdr:row>10</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -862,7 +862,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Opsional — biasanya cukup unggah foto ke folder foto Drive dengan nama yang sesuai (lihat tab petunjuk). Isi kolom ini hanya untuk menimpanya dengan tautan berbagi satu foto.
+          <t xml:space="preserve">Diisi otomatis lewat menu Situs → Pasang / ganti foto (pilih barisnya dulu). Kosong = foto bawaan situs.
 Contoh: https://drive.google.com/file/d/…/view</t>
         </r>
       </text>
@@ -880,7 +880,7 @@
                 <xdr:col>4</xdr:col>
                 <xdr:colOff>-367</xdr:colOff>
                 <xdr:row>2</xdr:row>
-                <xdr:rowOff>108</xdr:rowOff>
+                <xdr:rowOff>4</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1562,7 +1562,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Tautan satu foto Drive — atau kosongkan dan unggah foto ke folder Drive galeri/ dengan nama berkas = judul.
+          <t xml:space="preserve">WAJIB untuk galeri. Pilih baris ini lalu menu Situs → Pasang / ganti foto.
 Contoh: https://drive.google.com/file/d/…/view</t>
         </r>
       </text>
@@ -1579,8 +1579,8 @@
               <xdr:to>
                 <xdr:col>4</xdr:col>
                 <xdr:colOff>32</xdr:colOff>
-                <xdr:row>10</xdr:row>
-                <xdr:rowOff>16</xdr:rowOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>3</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1627,7 +1627,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="387">
   <si>
     <t xml:space="preserve">PETUNJUK MENGELOLA DATA — Website Kelurahan Lahendong</t>
   </si>
@@ -1659,37 +1659,22 @@
     <t xml:space="preserve">• Setelah mengubah data, buka halaman Cek Data: https://vercoooo.github.io/web-lahendong/cek-data.html — setiap isian yang keliru ditunjukkan beserta cara memperbaikinya.</t>
   </si>
   <si>
-    <t xml:space="preserve">FOTO DARI GOOGLE DRIVE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cara utama: unggah foto ke folder "Foto Situs Lahendong" di Google Drive (menu Situs → Buka folder foto). Situs mengenali foto dari NAMA BERKAS dan SUBFOLDER-nya:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• beranda/hero.jpg → gambar besar di Beranda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• wisata/&lt;nama destinasi&gt;.jpg → mis. wisata/Danau Linow.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• aparat/&lt;jabatan atau nama tanpa gelar&gt;.jpg → mis. aparat/Lurah.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• lingkungan/&lt;nama kepala/wakil&gt;.jpg → mis. lingkungan/Julius Joni Rondonuwu.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• kkt/&lt;NIM atau nama&gt;.jpg → mis. kkt/230211060074.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• galeri/&lt;kategori&gt;/&lt;judul&gt;.jpg → setiap foto otomatis masuk Galeri, mis. galeri/Kegiatan/Panen Raya.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mengganti foto: hapus berkas lama, unggah yang baru dengan nama sama. Menghapus: hapus berkasnya. Huruf besar/kecil dan ekstensi (.jpg/.png/.webp) bebas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perubahan tampil paling lambat 10 menit kemudian, atau segera lewat menu Situs → Sinkronkan foto sekarang. Foto orang 3:4 (pas foto), lanskap 3:2; hanya dengan izin yang bersangkutan.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kolom foto di tab lain (tautan Drive satu foto) tetap bisa dipakai untuk menimpa foto dari folder. Cek Data menandai nama berkas yang tidak cocok dengan data mana pun.</t>
+    <t xml:space="preserve">MEMASANG FOTO (menu Situs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Klik baris yang ingin diberi foto (tab wisata, aparat, galeri, atau baris foto_hero di tab profil).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Menu Situs → Pasang / ganti foto…  (panel muncul di samping kanan).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Pilih foto → Simpan foto. Selesai — tautannya ditulis otomatis ke kolom foto. Muat ulang halaman situs untuk melihatnya.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Melepas foto: buka panel yang sama → Hapus foto dari baris ini. Situs kembali memakai gambar bawaan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Panel hanya ada di Google Sheets versi komputer (browser). Foto orang hanya dengan izin yang bersangkutan.</t>
   </si>
   <si>
     <t xml:space="preserve">TAB</t>
@@ -1761,16 +1746,7 @@
     <t xml:space="preserve">Galeri</t>
   </si>
   <si>
-    <t xml:space="preserve">Opsional: judul &amp; kategori lewat sheet. Foto di folder Drive galeri/ sudah otomatis masuk Galeri tanpa baris di sini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">foto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Semua halaman yang berfoto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diisi OTOMATIS dari folder foto Google Drive oleh skrip (menu Situs). Jangan diedit.</t>
+    <t xml:space="preserve">Foto tambahan (kegiatan, alam, budaya) selain foto wisata</t>
   </si>
   <si>
     <t xml:space="preserve">ATURAN PENGISIAN</t>
@@ -1959,7 +1935,7 @@
     <t xml:space="preserve">aparat · foto</t>
   </si>
   <si>
-    <t xml:space="preserve">Opsional — biasanya cukup unggah foto ke folder foto Drive dengan nama yang sesuai (lihat tab petunjuk). Isi kolom ini hanya untuk menimpanya dengan tautan berbagi satu foto.</t>
+    <t xml:space="preserve">Diisi otomatis lewat menu Situs → Pasang / ganti foto (pilih barisnya dulu). Kosong = foto bawaan situs.</t>
   </si>
   <si>
     <t xml:space="preserve">https://drive.google.com/file/d/…/view</t>
@@ -2187,7 +2163,7 @@
     <t xml:space="preserve">galeri · foto</t>
   </si>
   <si>
-    <t xml:space="preserve">Tautan satu foto Drive — atau kosongkan dan unggah foto ke folder Drive galeri/ dengan nama berkas = judul.</t>
+    <t xml:space="preserve">WAJIB untuk galeri. Pilih baris ini lalu menu Situs → Pasang / ganti foto.</t>
   </si>
   <si>
     <t xml:space="preserve">galeri · kategori</t>
@@ -2580,6 +2556,9 @@
   </si>
   <si>
     <t xml:space="preserve">nomor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">foto</t>
   </si>
   <si>
     <t xml:space="preserve">Sekretaris Kelurahan</t>
@@ -3168,7 +3147,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28.6"/>
@@ -3237,22 +3216,22 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
@@ -3262,675 +3241,688 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+      <c r="B20" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C20" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>22</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2"/>
+        <v>25</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2"/>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B32" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C32" s="2" t="s">
+    </row>
+    <row r="33" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
+    <row r="34" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="2" t="s">
+    </row>
+    <row r="35" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C33" s="2" t="s">
+    </row>
+    <row r="36" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="2" t="s">
         <v>47</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2"/>
-    </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
+    <row r="40" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2" t="s">
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2"/>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2" t="s">
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="3" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="41" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="2" t="s">
+      <c r="B43" s="3" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="42" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="2" t="s">
+      <c r="C43" s="3" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="2" t="s">
+    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="44" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="2" t="s">
+      <c r="B44" s="4" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C44" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>59</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="2"/>
+      <c r="A47" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>66</v>
+      <c r="A48" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>75</v>
+      <c r="A53" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>81</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>96</v>
+      <c r="A60" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B61" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C61" s="4" t="s">
-        <v>99</v>
+      <c r="A61" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="C64" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B66" s="2" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="2" t="s">
+      <c r="C66" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B65" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="B66" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="C66" s="4" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B71" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="C71" s="4" t="s">
-        <v>129</v>
+      <c r="A71" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>116</v>
+        <v>137</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>111</v>
+        <v>141</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="C77" s="2" t="s">
-        <v>143</v>
+      <c r="A77" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>145</v>
+        <v>108</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>146</v>
+        <v>109</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="B83" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="C83" s="4" t="s">
-        <v>161</v>
+      <c r="A83" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>116</v>
+        <v>171</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>117</v>
+        <v>172</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>165</v>
+      <c r="A85" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>167</v>
+        <v>108</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>168</v>
+        <v>109</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>171</v>
+        <v>103</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="B89" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="C89" s="2" t="s">
-        <v>177</v>
-      </c>
+      <c r="A89" s="2"/>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>180</v>
+      <c r="A90" s="3" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="B91" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="C91" s="4" t="s">
+      <c r="A91" s="3" t="s">
         <v>183</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3938,214 +3930,165 @@
         <v>184</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="C92" s="2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="93" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="C93" s="2" t="s">
-        <v>111</v>
+        <v>187</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="C94" s="2" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="2"/>
+      <c r="A95" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="3" t="s">
-        <v>190</v>
+      <c r="A96" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="B97" s="3" t="s">
-        <v>23</v>
+      <c r="A97" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>66</v>
+        <v>201</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="B108" s="2" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="2"/>
+    </row>
+    <row r="108" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="3" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="B109" s="2" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B110" s="2" t="s">
+    </row>
+    <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="2"/>
+    </row>
+    <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="3" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="2" t="s">
+    <row r="113" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B111" s="2" t="s">
+    </row>
+    <row r="114" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="2" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="2" t="s">
+    <row r="115" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="2" t="s">
         <v>219</v>
-      </c>
-      <c r="B112" s="2" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="2"/>
-    </row>
-    <row r="114" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="3" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="115" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="2" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="2"/>
-    </row>
-    <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="3" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="119" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="2" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="120" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="2" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="121" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="2" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="122" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="2" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -4173,172 +4116,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4871,232 +4814,232 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6126,27 +6069,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>45</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="2"/>
@@ -6154,26 +6097,26 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -6912,70 +6855,70 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7718,144 +7661,144 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>45</v>
+        <v>309</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>333</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>334</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>335</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>336</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>338</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>339</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>342</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>343</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>345</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>346</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>347</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>352</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>355</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>357</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>358</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2" t="s">
-        <v>367</v>
+        <v>360</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9296,149 +9239,149 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>370</v>
+        <v>363</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>376</v>
+        <v>369</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="H2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>379</v>
+        <v>372</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>380</v>
+        <v>373</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>383</v>
+        <v>376</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>384</v>
+        <v>377</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="H4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>385</v>
+        <v>378</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>386</v>
+        <v>379</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>387</v>
+        <v>380</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>388</v>
+        <v>381</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>389</v>
+        <v>382</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="H5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>390</v>
+        <v>383</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>392</v>
+        <v>385</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="H6" s="2"/>
     </row>
@@ -10477,16 +10420,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>45</v>
+        <v>309</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
feat: kontak & galeri tanpa sel kosong, jam layanan per hari, refaktor kode foto
- Kontak: 2 kolom, jumlah ganjil membuat kartu pertama (mis. Lurah) satu baris penuh
- Galeri wisata: baris rata kiri-kanan mengikuti rasio foto (potret tidak terpotong);
  judul "Suasana" diganti "Galeri — Foto & video …"
- Jam layanan per kelompok hari (dipisah /): daftar hari–jam, bilah atas menampilkan jam hari ini
- DESTINASI & FOTO_ORANG menggantikan FOTO/MEDIA_DESTINASI; media tiap destinasi di img/wisata/<kode>/
- Hapus kode mati: pembaca tautan Drive, rantai foto cadangan, kalimatPertama, opsi opsional,
  URL_SHEET, CSS rata-kiri/data-hp/eyebrow-terang, gambar toulangkow

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/template-data-lahendong.xlsx
+++ b/data/template-data-lahendong.xlsx
@@ -56,8 +56,8 @@
               <xdr:to>
                 <xdr:col>2</xdr:col>
                 <xdr:colOff>-367</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>10</xdr:rowOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>12</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -74,7 +74,7 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">Isi informasinya. Beberapa paragraf: pisahkan dengan baris baru (Ctrl+Enter).
-Contoh: Senin – Jumat, 08.00 – 15.00 WITA</t>
+Contoh: Senin – Kamis, 08.00 – 16.30 WITA / Jumat, 08.00 – 13.30 WITA</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -90,8 +90,8 @@
               <xdr:to>
                 <xdr:col>3</xdr:col>
                 <xdr:colOff>-367</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+                <xdr:row>8</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1412,7 +1412,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="365">
   <si>
     <t xml:space="preserve">PETUNJUK MENGELOLA DATA — Website Kelurahan Lahendong</t>
   </si>
@@ -1582,7 +1582,7 @@
     <t xml:space="preserve">Isi informasinya. Beberapa paragraf: pisahkan dengan baris baru (Ctrl+Enter).</t>
   </si>
   <si>
-    <t xml:space="preserve">Senin – Jumat, 08.00 – 15.00 WITA</t>
+    <t xml:space="preserve">Senin – Kamis, 08.00 – 16.30 WITA / Jumat, 08.00 – 13.30 WITA</t>
   </si>
   <si>
     <t xml:space="preserve">profil · keterangan</t>
@@ -1930,7 +1930,7 @@
     <t xml:space="preserve">Email kantor</t>
   </si>
   <si>
-    <t xml:space="preserve">Jam layanan kantor</t>
+    <t xml:space="preserve">Jam layanan per kelompok hari, dipisah / — mis. Senin – Kamis, 08.00 – 16.30 WITA / Jumat, 08.00 – 13.30 WITA / Sabtu – Minggu, Tutup. Bilah atas situs menampilkan jam hari ini.</t>
   </si>
   <si>
     <t xml:space="preserve">luas_wilayah</t>
@@ -2036,6 +2036,9 @@
   </si>
   <si>
     <t xml:space="preserve">Halaman Kontak. Kosong = tidak ditampilkan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Senin – Kamis, 08.00 – 16.30 WITA / Jumat, 08.00 – 13.30 WITA / Sabtu – Minggu, Hanya keadaan mendesak</t>
   </si>
   <si>
     <t xml:space="preserve">CONTOH — ganti. Header, footer, halaman Kontak dan Layanan.</t>
@@ -3578,7 +3581,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
         <v>53</v>
       </c>
@@ -3775,15 +3778,15 @@
         <v>207</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>56</v>
+        <v>208</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3791,10 +3794,10 @@
         <v>173</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3802,10 +3805,10 @@
         <v>175</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3813,10 +3816,10 @@
         <v>177</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3824,10 +3827,10 @@
         <v>179</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3835,10 +3838,10 @@
         <v>181</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>217</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3846,10 +3849,10 @@
         <v>183</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3857,10 +3860,10 @@
         <v>185</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3868,10 +3871,10 @@
         <v>187</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3879,10 +3882,10 @@
         <v>189</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3890,10 +3893,10 @@
         <v>191</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4426,33 +4429,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>65</v>
@@ -4478,28 +4481,28 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4507,151 +4510,151 @@
         <v>62</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>242</v>
-      </c>
       <c r="E4" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5681,16 +5684,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5705,10 +5708,10 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>92</v>
@@ -5720,7 +5723,7 @@
         <v>86</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>92</v>
@@ -6361,70 +6364,70 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7167,37 +7170,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7208,97 +7211,97 @@
         <v>101</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8643,45 +8646,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>157</v>
@@ -8702,36 +8705,36 @@
         <v>148</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>160</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>157</v>
@@ -8743,22 +8746,22 @@
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>160</v>
@@ -8767,19 +8770,19 @@
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>157</v>

</xml_diff>

<commit_message>
fix: destinasi "Air Panas Belerang dan Hutan Pinus" kembali tampil
Nama di sheet diganti admin dari "Objek Wisata Air Panas Belerang dan Hutan Pinus" menjadi
"Air Panas Belerang dan Hutan Pinus", sehingga kodenya tidak lagi cocok dengan DESTINASI dan
barisnya dibuang wisataTetap() (Wisata, Beranda, dan detail).

- Kode DESTINASI & folder foto: air-panas-belerang-dan-hutan-pinus (mengikuti nama di sheet)
- data-contoh.js & template .xlsx: dropdown nama memuat nama baru
- wisata-detail.js: KODE_LAMA mengarahkan tautan ?id= lama ke destinasi yang sama

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RqTa7uQfJELZ19R5bSiHDn
</commit_message>
<xml_diff>
--- a/data/template-data-lahendong.xlsx
+++ b/data/template-data-lahendong.xlsx
@@ -2589,7 +2589,7 @@
     <t xml:space="preserve">https://maps.google.com/?q=Danau+Linow+Tomohon</t>
   </si>
   <si>
-    <t xml:space="preserve">Objek Wisata Air Panas Belerang dan Hutan Pinus</t>
+    <t xml:space="preserve">Air Panas Belerang dan Hutan Pinus</t>
   </si>
   <si>
     <t xml:space="preserve">Hutan pinus sejuk yang berpadu dengan kolam sulfur beruap putih.</t>
@@ -7899,7 +7899,7 @@
   <dimension ref="A1:K104"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="55.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="67.41"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="53.93"/>
@@ -9343,7 +9343,7 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation allowBlank="true" error="Pilih salah satu dari daftar." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A104" type="list">
-      <formula1>"Danau Linow,Objek Wisata Air Panas Belerang dan Hutan Pinus,Mah’Watu"</formula1>
+      <formula1>"Danau Linow,Air Panas Belerang dan Hutan Pinus,Mah’Watu"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Pilih salah satu dari daftar." errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B104" type="list">

</xml_diff>

<commit_message>
chore: siap pindah ke kelurahan-lahendong.github.io
- Kode situs tidak berubah: semua path aset & tautan internal sudah relatif, tidak ada path
  absolut, canonical/og:url, maupun build Tailwind (CDN); diuji jalan di akar domain dan di
  sub-folder /web-lahendong/
- README, Panduan Teknis, tools/buat_template.py (ALAMAT_SITUS) → https://kelurahan-lahendong.github.io/;
  template .xlsx dibuat ulang (tab petunjuk memuat alamat Cek Data yang baru)
- tools/pengalihan-url-lama/: index.html + 404.html untuk repo "web-lahendong" di akun lama, meneruskan
  setiap alamat lama ke halaman yang sama di alamat baru (?id dan #hash dipertahankan)
- URL Google Sheets dan layanan eksternal tidak diubah

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RqTa7uQfJELZ19R5bSiHDn
</commit_message>
<xml_diff>
--- a/data/template-data-lahendong.xlsx
+++ b/data/template-data-lahendong.xlsx
@@ -1520,7 +1520,7 @@
     <t xml:space="preserve">• Angka total (jumlah penduduk, KK, jiwa per lingkungan) tidak perlu ditulis — situs menghitungnya dari tab lingkungan.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Setelah mengubah data, buka halaman Cek Data: https://vercoooo.github.io/web-lahendong/cek-data.html — setiap isian yang keliru ditunjukkan beserta cara memperbaikinya.</t>
+    <t xml:space="preserve">• Setelah mengubah data, buka halaman Cek Data: https://kelurahan-lahendong.github.io/cek-data.html — setiap isian yang keliru ditunjukkan beserta cara memperbaikinya.</t>
   </si>
   <si>
     <t xml:space="preserve">FOTO &amp; DESTINASI WISATA</t>
@@ -3073,7 +3073,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>

</xml_diff>